<commit_message>
login book Store App using Data Driven Tetsting
</commit_message>
<xml_diff>
--- a/src/test/Resources/Data Driven Testing File.xlsx
+++ b/src/test/Resources/Data Driven Testing File.xlsx
@@ -5,23 +5,25 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd36ce00b62d46e0/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\IdeaProjects\DemoQAHybridFramework\src\test\Resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{75270B39-794C-427E-8196-A6DB719D9192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A570ECB9-C9E6-46D0-A6AE-52A17AEED5AA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E76CB4C5-B111-432C-A6A5-F7A5B290ADA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="8964" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
     <sheet name="DemoQATestDataSheet" sheetId="2" r:id="rId2"/>
+    <sheet name="loginValidData" sheetId="3" r:id="rId3"/>
+    <sheet name="loginInValidData" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="36">
   <si>
     <t>Login ID</t>
   </si>
@@ -112,12 +114,42 @@
   <si>
     <t>ten</t>
   </si>
+  <si>
+    <t xml:space="preserve">name </t>
+  </si>
+  <si>
+    <t>jitendra</t>
+  </si>
+  <si>
+    <t>Callme@jithu123</t>
+  </si>
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ncx </t>
+  </si>
+  <si>
+    <t>vxckn</t>
+  </si>
+  <si>
+    <t>knjcnx</t>
+  </si>
+  <si>
+    <t>fvvjvf</t>
+  </si>
+  <si>
+    <t>hjd</t>
+  </si>
+  <si>
+    <t>vjbkd</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -128,6 +160,22 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -156,14 +204,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -687,4 +739,82 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68D469A3-4BE3-4214-A04C-A41144E4C394}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="16.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{7E93C917-C456-4E8C-88B4-49151607086F}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F73DE6D-0B17-4495-9C44-EF431FF4BC61}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.21875" customWidth="1"/>
+    <col min="2" max="2" width="18.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>